<commit_message>
Coverage QC: assigned-reading sections now taught in L01/L02 (signaling mechanisms, ionization/pKa, drug bonds and chirality, trial design and law, extraction ratio, dosing regimens, MFO system, diet/microbiota, OCT1/SLCO1B1/ABCG2, G6PD); audit gains reading-coverage gate, faculty-identifier policy, question checks now gate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016g9Y35CWfsLvVnVtnzR7rF
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit1_L01.xlsx
+++ b/docs/sketch/kahoot/unit1_L01.xlsx
@@ -1589,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA141"/>
+  <dimension ref="A1:AA151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="12.5" customWidth="1" min="1" max="1"/>
@@ -6891,17 +6891,17 @@
       </c>
       <c r="C97" s="16" t="inlineStr">
         <is>
-          <t>Phase I</t>
+          <t>FDA review</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>FDA review</t>
+          <t>Phase III</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Phase III</t>
+          <t>Phase IV</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
@@ -6943,27 +6943,27 @@
       </c>
       <c r="B98" s="16" t="inlineStr">
         <is>
-          <t>Pharmacology: which is right?</t>
+          <t>A drug activates a receptor coupled to Gq. Which change follows inside the cell?</t>
         </is>
       </c>
       <c r="C98" s="16" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Phospholipase C makes IP₃ and DAG; calcium rises</t>
         </is>
       </c>
       <c r="D98" s="16" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>Adenylyl cyclase is stimulated, so cAMP rises</t>
         </is>
       </c>
       <c r="E98" s="16" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Phosphodiesterase breaks down cGMP in the cell</t>
         </is>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Adenylyl cyclase is inhibited, so cAMP falls</t>
         </is>
       </c>
       <c r="G98" s="14" t="n">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="H98" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I98" s="1" t="n"/>
@@ -7000,27 +7000,27 @@
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Pharmacologic vs. therapeutic effect: which is right?</t>
+          <t>A patient overdoses on a weak-acid drug. To speed its renal excretion, what should be done to the urine?</t>
         </is>
       </c>
       <c r="C99" s="16" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Keep urine pH unchanged and give more fluids only</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Any measurable biological change vs. the intended, beneficial effect</t>
+          <t>Make the urine more acidic</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Raise plasma protein binding</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Make the urine more alkaline</t>
         </is>
       </c>
       <c r="G99" s="14" t="n">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="H99" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I99" s="1" t="n"/>
@@ -7057,27 +7057,27 @@
       </c>
       <c r="B100" s="16" t="inlineStr">
         <is>
-          <t>Adverse drug reaction (ADR): which is right?</t>
+          <t>Pharmacology: which is right?</t>
         </is>
       </c>
       <c r="C100" s="16" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="D100" s="16" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="G100" s="14" t="n">
@@ -7114,27 +7114,27 @@
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Toxicity: which is right?</t>
+          <t>Pharmacologic vs. therapeutic effect: which is right?</t>
         </is>
       </c>
       <c r="C101" s="16" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Any measurable biological change vs. the intended, beneficial effect</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G101" s="14" t="n">
@@ -7171,27 +7171,27 @@
       </c>
       <c r="B102" s="16" t="inlineStr">
         <is>
-          <t>Why prescribe by generic name: which is right?</t>
+          <t>Adverse drug reaction (ADR): which is right?</t>
         </is>
       </c>
       <c r="C102" s="16" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="D102" s="16" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="G102" s="14" t="n">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="H102" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I102" s="1" t="n"/>
@@ -7228,31 +7228,31 @@
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Tylenol: which is right?</t>
+          <t>Toxicity: which is right?</t>
         </is>
       </c>
       <c r="C103" s="16" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="G103" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H103" s="18" t="inlineStr">
         <is>
@@ -7285,27 +7285,27 @@
       </c>
       <c r="B104" s="16" t="inlineStr">
         <is>
-          <t>Pharmacokinetics vs. pharmacodynamics: which is right?</t>
+          <t>Why prescribe by generic name: which is right?</t>
         </is>
       </c>
       <c r="C104" s="16" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="D104" s="16" t="inlineStr">
         <is>
-          <t>Applying PK/PD to real patients; the study of poisoning</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E104" s="16" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="F104" s="16" t="inlineStr">
         <is>
-          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="G104" s="14" t="n">
@@ -7313,7 +7313,7 @@
       </c>
       <c r="H104" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I104" s="1" t="n"/>
@@ -7342,35 +7342,35 @@
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Pharmacogenomics: which is right?</t>
+          <t>Tylenol: which is right?</t>
         </is>
       </c>
       <c r="C105" s="16" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>pH where ionized = nonionized</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Randomized controlled trial</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Brand name of acetaminophen</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Natural ligand unknown</t>
         </is>
       </c>
       <c r="G105" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H105" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I105" s="1" t="n"/>
@@ -7399,35 +7399,35 @@
       </c>
       <c r="B106" s="16" t="inlineStr">
         <is>
-          <t>Clinical pharmacology / toxicology: which is right?</t>
+          <t>Pharmacokinetics vs. pharmacodynamics: which is right?</t>
         </is>
       </c>
       <c r="C106" s="16" t="inlineStr">
         <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="inlineStr">
+        <is>
           <t>Applying PK/PD to real patients; the study of poisoning</t>
         </is>
       </c>
-      <c r="D106" s="16" t="inlineStr">
-        <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
-        </is>
-      </c>
       <c r="E106" s="16" t="inlineStr">
         <is>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+        </is>
+      </c>
+      <c r="F106" s="16" t="inlineStr">
+        <is>
           <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
         </is>
       </c>
-      <c r="F106" s="16" t="inlineStr">
-        <is>
-          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
-        </is>
-      </c>
       <c r="G106" s="14" t="n">
         <v>30</v>
       </c>
       <c r="H106" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I106" s="1" t="n"/>
@@ -7456,27 +7456,27 @@
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>4 sources of new drugs: which is right?</t>
+          <t>Pharmacogenomics: which is right?</t>
         </is>
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="G107" s="14" t="n">
@@ -7484,7 +7484,7 @@
       </c>
       <c r="H107" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I107" s="1" t="n"/>
@@ -7513,27 +7513,27 @@
       </c>
       <c r="B108" s="16" t="inlineStr">
         <is>
-          <t>Biologics: which is right?</t>
+          <t>Clinical pharmacology / toxicology: which is right?</t>
         </is>
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Applying PK/PD to real patients; the study of poisoning</t>
         </is>
       </c>
       <c r="D108" s="16" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
         </is>
       </c>
       <c r="F108" s="16" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
         </is>
       </c>
       <c r="G108" s="14" t="n">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="H108" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I108" s="1" t="n"/>
@@ -7570,35 +7570,35 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Phase I: which is right?</t>
+          <t>4 sources of new drugs: which is right?</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
           <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
-        </is>
-      </c>
       <c r="G109" t="n">
         <v>30</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -7608,27 +7608,27 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Phase III: which is right?</t>
+          <t>Biologics: which is right?</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G110" t="n">
@@ -7636,7 +7636,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7646,27 +7646,27 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Phase IV: which is right?</t>
+          <t>Phase I: which is right?</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="G111" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -7684,27 +7684,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Rare AE (1 in 10,000): which is right?</t>
+          <t>Phase III: which is right?</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -7722,27 +7722,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Efficacy vs. effectiveness: which is right?</t>
+          <t>Phase IV: which is right?</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Postmarketing surveillance — general prescribed population</t>
         </is>
       </c>
       <c r="G113" t="n">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7760,27 +7760,27 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>FDA MedWatch: which is right?</t>
+          <t>Rare AE (1 in 10,000): which is right?</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
           <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
+      <c r="F114" t="inlineStr">
         <is>
           <t>Often first found in Phase IV — trials too small/short</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Adverse-event reporting system (voluntary + mandatory)</t>
         </is>
       </c>
       <c r="G114" t="n">
@@ -7798,27 +7798,27 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Risk-benefit case: 70% improve, 1% serious hepatotoxicity: which is right?</t>
+          <t>Efficacy vs. effectiveness: which is right?</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="G115" t="n">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -7836,27 +7836,27 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>5 drug target classes: which is right?</t>
+          <t>FDA MedWatch: which is right?</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>Adverse-event reporting system (voluntary + mandatory)</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -7874,27 +7874,27 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Receptor types: which is right?</t>
+          <t>Risk-benefit case: 70% improve, 1% serious hepatotoxicity: which is right?</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7912,27 +7912,27 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Most common targets: which is right?</t>
+          <t>5 drug target classes: which is right?</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
         </is>
       </c>
       <c r="G118" t="n">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7950,27 +7950,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Competitive antagonist: which is right?</t>
+          <t>Receptor types: which is right?</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="G119" t="n">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -7988,27 +7988,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Potency: which is right?</t>
+          <t>Most common targets: which is right?</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ANDA with bioequivalence data; patent life 20 years</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="G120" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8026,27 +8026,27 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EC₅₀: which is right?</t>
+          <t>Competitive antagonist: which is right?</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="G121" t="n">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8064,27 +8064,27 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Therapeutic index: which is right?</t>
+          <t>Potency: which is right?</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>ANDA with bioequivalence data; patent life 20 years</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="G122" t="n">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8102,35 +8102,35 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Narrow-TI drugs: which is right?</t>
+          <t>EC₅₀: which is right?</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="G123" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8140,27 +8140,27 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Bioavailability (F): which is right?</t>
+          <t>Therapeutic index: which is right?</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8178,35 +8178,35 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Why oral F &lt; 100%: which is right?</t>
+          <t>Narrow-TI drugs: which is right?</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8216,24 +8216,24 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>First-pass path: which is right?</t>
+          <t>Bioavailability (F): which is right?</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
           <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
-        </is>
-      </c>
       <c r="F126" t="inlineStr">
         <is>
           <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
@@ -8244,7 +8244,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8254,27 +8254,27 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Big first-pass drugs: which is right?</t>
+          <t>Why oral F &lt; 100%: which is right?</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8292,27 +8292,27 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sublingual: which is right?</t>
+          <t>First-pass path: which is right?</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="G128" t="n">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8330,27 +8330,27 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>IM / SC / transdermal: which is right?</t>
+          <t>Big first-pass drugs: which is right?</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="G129" t="n">
@@ -8368,27 +8368,27 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Inhaled / topical: which is right?</t>
+          <t>Sublingual: which is right?</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="G130" t="n">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8406,27 +8406,27 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Plasma protein binding: which is right?</t>
+          <t>IM / SC / transdermal: which is right?</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="G131" t="n">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8444,27 +8444,27 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tissue perfusion: which is right?</t>
+          <t>Inhaled / topical: which is right?</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G132" t="n">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Polar antibiotic + meningitis: which is right?</t>
+          <t>Plasma protein binding: which is right?</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -8492,25 +8492,25 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
           <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
-        </is>
-      </c>
       <c r="G133" t="n">
         <v>30</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8520,27 +8520,27 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Phase I size (textbook): which is right?</t>
+          <t>Tissue perfusion: which is right?</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G134" t="n">
@@ -8558,31 +8558,31 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Phase with highest failure: which is right?</t>
+          <t>Polar antibiotic + meningitis: which is right?</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Postmarketing surveillance — general prescribed population</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -8596,27 +8596,27 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Kefauver-Harris (1962): which is right?</t>
+          <t>Phase I size (textbook): which is right?</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Protamine neutralizes heparin — no receptor</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="G136" t="n">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8634,35 +8634,35 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Generic approval: which is right?</t>
+          <t>Phase with highest failure: which is right?</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ANDA with bioequivalence data; patent life 20 years</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8672,27 +8672,27 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Spare receptors: which is right?</t>
+          <t>Kefauver-Harris (1962): which is right?</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Protamine neutralizes heparin — no receptor</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="G138" t="n">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8710,27 +8710,27 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Chemical antagonist: which is right?</t>
+          <t>Generic approval: which is right?</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Protamine neutralizes heparin — no receptor</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>ANDA with bioequivalence data; patent life 20 years</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G139" t="n">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8748,27 +8748,27 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Therapeutic window: which is right?</t>
+          <t>Spare receptors: which is right?</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G140" t="n">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8786,33 +8786,413 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
+          <t>Chemical antagonist: which is right?</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Protamine neutralizes heparin — no receptor</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Always comparative — "compared to what?"</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Phase II — only ~25% move to Phase III</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Required proof of efficacy (thalidomide)</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>30</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>134</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Therapeutic window: which is right?</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>30</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>135</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
           <t>Aspirin overdose: which is right?</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C143" t="inlineStr">
         <is>
           <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
         </is>
       </c>
-      <c r="D141" t="inlineStr">
+      <c r="D143" t="inlineStr">
         <is>
           <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
+      <c r="E143" t="inlineStr">
         <is>
           <t>Adverse-event reporting system (voluntary + mandatory)</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr">
+      <c r="F143" t="inlineStr">
         <is>
           <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
-      <c r="G141" t="n">
-        <v>30</v>
-      </c>
-      <c r="H141" t="inlineStr">
+      <c r="G143" t="n">
+        <v>30</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>136</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Most drugs’ molecular weight: which is right?</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Natural ligand unknown</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>~100–1000</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>20</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>137</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Weak bonds vs covalent: which is right?</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>30</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>138</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>pKa: which is right?</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>20</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>139</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Ion trapping: which is right?</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Postmarketing surveillance — general prescribed population</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>30</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>140</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Intracellular receptors: which is right?</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>30</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>141</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Gs / Gi / Gq: which is right?</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Phase II — only ~25% move to Phase III</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>20</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>142</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Gold-standard trial: which is right?</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Natural ligand unknown</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="G150" t="n">
+        <v>20</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>143</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Orphan receptor: which is right?</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Natural ligand unknown</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>20</v>
+      </c>
+      <c r="H151" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>

<commit_message>
QC: browser-wide and data-wide checks join ./run.sh check; reusable interactive figure types (dose-response, antagonist, bars, half-life, steady-state …) so new lectures' figures get hands-on versions; 25 more self-test questions fit Kahoot
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016g9Y35CWfsLvVnVtnzR7rF
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit1_L01.xlsx
+++ b/docs/sketch/kahoot/unit1_L01.xlsx
@@ -1589,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA151"/>
+  <dimension ref="A1:AA161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="12.5" customWidth="1" min="1" max="1"/>
@@ -6886,17 +6886,17 @@
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>According to the textbook, which clinical trial phase has the highest rate of drug failures?</t>
+          <t>Which trial phase first tests a drug in a large patient population to confirm efficacy just before approval?</t>
         </is>
       </c>
       <c r="C97" s="16" t="inlineStr">
         <is>
-          <t>FDA review</t>
+          <t>Phase III</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Phase III</t>
+          <t>Phase II</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Phase II</t>
+          <t>Phase I</t>
         </is>
       </c>
       <c r="G97" s="14" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="H97" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I97" s="1" t="n"/>
@@ -6943,27 +6943,27 @@
       </c>
       <c r="B98" s="16" t="inlineStr">
         <is>
-          <t>A drug activates a receptor coupled to Gq. Which change follows inside the cell?</t>
+          <t>A drug at the agonist’s receptor lowers baseline (constitutive) activity with no agonist present. It is a(n):</t>
         </is>
       </c>
       <c r="C98" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase C makes IP₃ and DAG; calcium rises</t>
+          <t>Inverse agonist</t>
         </is>
       </c>
       <c r="D98" s="16" t="inlineStr">
         <is>
-          <t>Adenylyl cyclase is stimulated, so cAMP rises</t>
+          <t>Full agonist</t>
         </is>
       </c>
       <c r="E98" s="16" t="inlineStr">
         <is>
-          <t>Phosphodiesterase breaks down cGMP in the cell</t>
+          <t>Partial agonist</t>
         </is>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
-          <t>Adenylyl cyclase is inhibited, so cAMP falls</t>
+          <t>Competitive antagonist</t>
         </is>
       </c>
       <c r="G98" s="14" t="n">
@@ -7000,27 +7000,27 @@
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>A patient overdoses on a weak-acid drug. To speed its renal excretion, what should be done to the urine?</t>
+          <t>Drug X needs a lower dose than Drug Y for the same effect; both reach the same Emax. Which is correct?</t>
         </is>
       </c>
       <c r="C99" s="16" t="inlineStr">
         <is>
-          <t>Keep urine pH unchanged and give more fluids only</t>
+          <t>Drug X is more potent than Drug Y</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Make the urine more acidic</t>
+          <t>Drug X is more efficacious than Drug Y</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Raise plasma protein binding</t>
+          <t>Drug X and Drug Y have different Emax values</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Make the urine more alkaline</t>
+          <t>Drug X has a narrower therapeutic index than Drug Y</t>
         </is>
       </c>
       <c r="G99" s="14" t="n">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="H99" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I99" s="1" t="n"/>
@@ -7057,27 +7057,27 @@
       </c>
       <c r="B100" s="16" t="inlineStr">
         <is>
-          <t>Pharmacology: which is right?</t>
+          <t>Which route bypasses first-pass hepatic metabolism by entering systemic venous circulation directly?</t>
         </is>
       </c>
       <c r="C100" s="16" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Oral, taken with food</t>
         </is>
       </c>
       <c r="D100" s="16" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>All routes undergo first-pass metabolism equally</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Sublingual</t>
         </is>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Oral, taken on an empty stomach</t>
         </is>
       </c>
       <c r="G100" s="14" t="n">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="H100" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I100" s="1" t="n"/>
@@ -7114,27 +7114,27 @@
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Pharmacologic vs. therapeutic effect: which is right?</t>
+          <t>Drug levels are in the therapeutic range, yet an unintended harmful response occurs. Which term fits?</t>
         </is>
       </c>
       <c r="C101" s="16" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Irreversible antagonism, because the receptor was permanently inactivated</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Any measurable biological change vs. the intended, beneficial effect</t>
+          <t>An adverse drug reaction, because it occurred at a normal therapeutic dose</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>A pharmacologic effect only, because it was a measurable biological change</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Toxicity, because any harmful drug response counts as toxicity</t>
         </is>
       </c>
       <c r="G101" s="14" t="n">
@@ -7171,27 +7171,27 @@
       </c>
       <c r="B102" s="16" t="inlineStr">
         <is>
-          <t>Adverse drug reaction (ADR): which is right?</t>
+          <t>A drug worked in a controlled trial, but fewer clinic patients improve (missed doses, comorbidities). Why?</t>
         </is>
       </c>
       <c r="C102" s="16" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Competitive antagonism of the drug by the comorbid conditions</t>
         </is>
       </c>
       <c r="D102" s="16" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Real-world effectiveness falling below the drug's trial efficacy</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>A narrow therapeutic index that appeared after approval</t>
         </is>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Extensive first-pass metabolism in the clinic's patients</t>
         </is>
       </c>
       <c r="G102" s="14" t="n">
@@ -7228,35 +7228,35 @@
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Toxicity: which is right?</t>
+          <t>After approval, a 1-in-10,000 serious reaction appears that trials never showed. Why was it missed?</t>
         </is>
       </c>
       <c r="C103" s="16" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Adverse-event reporting systems accept only voluntary reports</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Approval came before the drug completed any clinical trial phase</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Phase III trials are not designed to monitor adverse effects</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Trial populations were too small and too short to detect so rare an event</t>
         </is>
       </c>
       <c r="G103" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H103" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I103" s="1" t="n"/>
@@ -7285,27 +7285,27 @@
       </c>
       <c r="B104" s="16" t="inlineStr">
         <is>
-          <t>Why prescribe by generic name: which is right?</t>
+          <t>According to the textbook, which clinical trial phase has the highest rate of drug failures?</t>
         </is>
       </c>
       <c r="C104" s="16" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>FDA review</t>
         </is>
       </c>
       <c r="D104" s="16" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Phase III</t>
         </is>
       </c>
       <c r="E104" s="16" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Phase IV</t>
         </is>
       </c>
       <c r="F104" s="16" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>Phase II</t>
         </is>
       </c>
       <c r="G104" s="14" t="n">
@@ -7313,7 +7313,7 @@
       </c>
       <c r="H104" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I104" s="1" t="n"/>
@@ -7342,31 +7342,31 @@
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Tylenol: which is right?</t>
+          <t>A receptor blocker’s effect is fully overcome by raising the agonist dose. The blocker is most likely a(n):</t>
         </is>
       </c>
       <c r="C105" s="16" t="inlineStr">
         <is>
-          <t>pH where ionized = nonionized</t>
+          <t>Noncompetitive antagonist</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Inverse agonist</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Competitive antagonist</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Natural ligand unknown</t>
+          <t>Irreversible antagonist</t>
         </is>
       </c>
       <c r="G105" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H105" s="18" t="inlineStr">
         <is>
@@ -7399,27 +7399,27 @@
       </c>
       <c r="B106" s="16" t="inlineStr">
         <is>
-          <t>Pharmacokinetics vs. pharmacodynamics: which is right?</t>
+          <t>An inhaled bronchodilator works in minutes; an oral corticosteroid takes hours. Why the steroid’s delay?</t>
         </is>
       </c>
       <c r="C106" s="16" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>It binds a G protein–coupled receptor that raises cAMP</t>
         </is>
       </c>
       <c r="D106" s="16" t="inlineStr">
         <is>
-          <t>Applying PK/PD to real patients; the study of poisoning</t>
+          <t>It acts on an intracellular receptor that changes gene transcription</t>
         </is>
       </c>
       <c r="E106" s="16" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>It must first be activated by CYP2D6</t>
         </is>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
-          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
+          <t>It acts on a ligand-gated ion channel</t>
         </is>
       </c>
       <c r="G106" s="14" t="n">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="H106" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I106" s="1" t="n"/>
@@ -7456,27 +7456,27 @@
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Pharmacogenomics: which is right?</t>
+          <t>A drug activates a receptor coupled to Gq. Which change follows inside the cell?</t>
         </is>
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Phospholipase C makes IP₃ and DAG; calcium rises</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Adenylyl cyclase is stimulated, so cAMP rises</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Phosphodiesterase breaks down cGMP in the cell</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Adenylyl cyclase is inhibited, so cAMP falls</t>
         </is>
       </c>
       <c r="G107" s="14" t="n">
@@ -7484,7 +7484,7 @@
       </c>
       <c r="H107" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I107" s="1" t="n"/>
@@ -7513,27 +7513,27 @@
       </c>
       <c r="B108" s="16" t="inlineStr">
         <is>
-          <t>Clinical pharmacology / toxicology: which is right?</t>
+          <t>A patient with meningitis gets a highly polar antibiotic. How well does it reach the CNS?</t>
         </is>
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>Applying PK/PD to real patients; the study of poisoning</t>
+          <t>Polar drugs cross easily because P-glycoprotein pumps them into the CNS</t>
         </is>
       </c>
       <c r="D108" s="16" t="inlineStr">
         <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
+          <t>Polar drugs never reach the CNS, even when the meninges are inflamed</t>
         </is>
       </c>
       <c r="E108" s="16" t="inlineStr">
         <is>
-          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
+          <t>Polar drugs cross easily because tight junctions favor polar molecules</t>
         </is>
       </c>
       <c r="F108" s="16" t="inlineStr">
         <is>
-          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+          <t>Polar drugs usually cross poorly, but inflamed meninges allow better entry</t>
         </is>
       </c>
       <c r="G108" s="14" t="n">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="H108" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I108" s="1" t="n"/>
@@ -7570,27 +7570,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>4 sources of new drugs: which is right?</t>
+          <t>A patient overdoses on a weak-acid drug. To speed its renal excretion, what should be done to the urine?</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Keep urine pH unchanged and give more fluids only</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+          <t>Make the urine more acidic</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Raise plasma protein binding</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Make the urine more alkaline</t>
         </is>
       </c>
       <c r="G109" t="n">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -7608,27 +7608,27 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Biologics: which is right?</t>
+          <t>Pharmacology: which is right?</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="G110" t="n">
@@ -7636,7 +7636,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -7646,27 +7646,27 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Phase I: which is right?</t>
+          <t>Pharmacologic vs. therapeutic effect: which is right?</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Any measurable biological change vs. the intended, beneficial effect</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G111" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -7684,27 +7684,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Phase III: which is right?</t>
+          <t>Adverse drug reaction (ADR): which is right?</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -7722,27 +7722,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Phase IV: which is right?</t>
+          <t>Toxicity: which is right?</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="G113" t="n">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -7760,27 +7760,27 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Rare AE (1 in 10,000): which is right?</t>
+          <t>Why prescribe by generic name: which is right?</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="G114" t="n">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -7798,31 +7798,31 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Efficacy vs. effectiveness: which is right?</t>
+          <t>Tylenol: which is right?</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
+          <t>pH where ionized = nonionized</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Randomized controlled trial</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Brand name of acetaminophen</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>Natural ligand unknown</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -7836,27 +7836,27 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>FDA MedWatch: which is right?</t>
+          <t>Pharmacokinetics vs. pharmacodynamics: which is right?</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Applying PK/PD to real patients; the study of poisoning</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -7874,27 +7874,27 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Risk-benefit case: 70% improve, 1% serious hepatotoxicity: which is right?</t>
+          <t>Pharmacogenomics: which is right?</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -7912,27 +7912,27 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>5 drug target classes: which is right?</t>
+          <t>Clinical pharmacology / toxicology: which is right?</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Applying PK/PD to real patients; the study of poisoning</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+          <t>Body → drug (ADME) vs. drug → body (receptors &amp; effect)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
         </is>
       </c>
       <c r="G118" t="n">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -7950,27 +7950,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Receptor types: which is right?</t>
+          <t>4 sources of new drugs: which is right?</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
           <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
+      <c r="F119" t="inlineStr">
         <is>
           <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="G119" t="n">
@@ -7988,27 +7988,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Most common targets: which is right?</t>
+          <t>Biologics: which is right?</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G120" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8026,27 +8026,27 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Competitive antagonist: which is right?</t>
+          <t>Phase I: which is right?</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
           <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="G121" t="n">
@@ -8064,27 +8064,27 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Potency: which is right?</t>
+          <t>Phase III: which is right?</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ANDA with bioequivalence data; patent life 20 years</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="G122" t="n">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8102,27 +8102,27 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EC₅₀: which is right?</t>
+          <t>Phase IV: which is right?</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+          <t>Postmarketing surveillance — general prescribed population</t>
         </is>
       </c>
       <c r="G123" t="n">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8140,27 +8140,27 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Therapeutic index: which is right?</t>
+          <t>Rare AE (1 in 10,000): which is right?</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Adverse-event reporting system (voluntary + mandatory)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8178,35 +8178,35 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Narrow-TI drugs: which is right?</t>
+          <t>Efficacy vs. effectiveness: which is right?</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8216,27 +8216,27 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Bioavailability (F): which is right?</t>
+          <t>FDA MedWatch: which is right?</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Often first found in Phase IV — trials too small/short</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Adverse-event reporting system (voluntary + mandatory)</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8254,27 +8254,27 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Why oral F &lt; 100%: which is right?</t>
+          <t>Risk-benefit case: 70% improve, 1% serious hepatotoxicity: which is right?</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Incomplete absorption + first-pass hepatic metabolism</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>How genetic variation shapes individual drug response</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="G127" t="n">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8292,27 +8292,27 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>First-pass path: which is right?</t>
+          <t>5 drug target classes: which is right?</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
         </is>
       </c>
       <c r="G128" t="n">
@@ -8330,27 +8330,27 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Big first-pass drugs: which is right?</t>
+          <t>Receptor types: which is right?</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="G129" t="n">
@@ -8368,27 +8368,27 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sublingual: which is right?</t>
+          <t>Most common targets: which is right?</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
+          <t>G-protein-coupled · ligand-gated ion channel · enzyme-linked · nuclear</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="G130" t="n">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8406,27 +8406,27 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>IM / SC / transdermal: which is right?</t>
+          <t>Competitive antagonist: which is right?</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="G131" t="n">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8444,27 +8444,27 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Inhaled / topical: which is right?</t>
+          <t>Potency: which is right?</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>ANDA with bioequivalence data; patent life 20 years</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="G132" t="n">
@@ -8482,27 +8482,27 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Plasma protein binding: which is right?</t>
+          <t>EC₅₀: which is right?</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="G133" t="n">
@@ -8510,7 +8510,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8520,27 +8520,27 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Tissue perfusion: which is right?</t>
+          <t>Therapeutic index: which is right?</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="G134" t="n">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8558,31 +8558,31 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Polar antibiotic + meningitis: which is right?</t>
+          <t>Narrow-TI drugs: which is right?</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
@@ -8596,27 +8596,27 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Phase I size (textbook): which is right?</t>
+          <t>Bioavailability (F): which is right?</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="G136" t="n">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8634,35 +8634,35 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Phase with highest failure: which is right?</t>
+          <t>Why oral F &lt; 100%: which is right?</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Incomplete absorption + first-pass hepatic metabolism</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>How genetic variation shapes individual drug response</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8672,27 +8672,27 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Kefauver-Harris (1962): which is right?</t>
+          <t>First-pass path: which is right?</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Protamine neutralizes heparin — no receptor</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="G138" t="n">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8710,27 +8710,27 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Generic approval: which is right?</t>
+          <t>Big first-pass drugs: which is right?</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ANDA with bioequivalence data; patent life 20 years</t>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="G139" t="n">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8748,27 +8748,27 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Spare receptors: which is right?</t>
+          <t>Sublingual: which is right?</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
+          <t>Directly into systemic venous circulation — skips portal vein &amp; liver</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
+          <t>Natural products · synthetic &amp; biotech · biologics · drug repurposing</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
+          <t>Safety, tolerability, dose-finding — small group of healthy volunteers</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
+          <t>Receptors and enzymes (ion channels/transporters: cardiac &amp; CNS drugs)</t>
         </is>
       </c>
       <c r="G140" t="n">
@@ -8786,27 +8786,27 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Chemical antagonist: which is right?</t>
+          <t>IM / SC / transdermal: which is right?</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Protamine neutralizes heparin — no receptor</t>
+          <t>Faster than oral, depot · slower steady (insulin, heparin) · slow sustained</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Always comparative — "compared to what?"</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Unambiguous, international; avoids hidden duplicate therapy (double-dosing)</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Required proof of efficacy (thalidomide)</t>
+          <t>Study of how drugs interact with living systems — molecule to whole patient</t>
         </is>
       </c>
       <c r="G141" t="n">
@@ -8824,27 +8824,27 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Therapeutic window: which is right?</t>
+          <t>Inhaled / topical: which is right?</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -8852,7 +8852,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8862,27 +8862,27 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Aspirin overdose: which is right?</t>
+          <t>Plasma protein binding: which is right?</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Often first found in Phase IV — trials too small/short</t>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="G143" t="n">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -8900,35 +8900,35 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Most drugs’ molecular weight: which is right?</t>
+          <t>Tissue perfusion: which is right?</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Natural ligand unknown</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>~100–1000</t>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G144" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -8938,27 +8938,27 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Weak bonds vs covalent: which is right?</t>
+          <t>Polar antibiotic + meningitis: which is right?</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+          <t>Postmarketing surveillance — general prescribed population</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
         </is>
       </c>
       <c r="G145" t="n">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -8976,35 +8976,35 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>pKa: which is right?</t>
+          <t>Phase I size (textbook): which is right?</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>20–100 healthy volunteers; patients if drug is very toxic (cancer, AIDS)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Confirm efficacy, monitor AEs at scale — hundreds to thousands, multi-site</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>pH where ionized = nonionized</t>
+          <t>Ideal trial conditions vs. everyday practice (adherence, comorbidities)</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+          <t>Same site, reversible, overcome by more agonist → curve right, same Emax</t>
         </is>
       </c>
       <c r="G146" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -9014,35 +9014,35 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Ion trapping: which is right?</t>
+          <t>Phase with highest failure: which is right?</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -9052,27 +9052,27 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Intracellular receptors: which is right?</t>
+          <t>Kefauver-Harris (1962): which is right?</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>Always comparative — "compared to what?"</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>Required proof of efficacy (thalidomide)</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+          <t>Protamine neutralizes heparin — no receptor</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="G148" t="n">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -9090,35 +9090,35 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Gs / Gi / Gq: which is right?</t>
+          <t>Generic approval: which is right?</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>pH where ionized = nonionized</t>
+          <t>Brain, heart, kidney get drug fast; fat, bone slowly</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>ANDA with bioequivalence data; patent life 20 years</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+          <t>Dose needed for an effect — lower EC₅₀ = more potent</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Monoclonal antibodies, gene- and cell-based therapies</t>
         </is>
       </c>
       <c r="G149" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -9128,35 +9128,35 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Gold-standard trial: which is right?</t>
+          <t>Spare receptors: which is right?</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>pH where ionized = nonionized</t>
+          <t>Max response without full occupancy (~90% cardiac β can be blocked)</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Natural ligand unknown</t>
+          <t>Oral → GI tract → portal circulation → liver → systemic circulation</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Fraction of dose reaching systemic circulation unchanged; IV = 100%</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Rapid local lung effect · local effect, minimal systemic absorption</t>
         </is>
       </c>
       <c r="G150" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -9166,33 +9166,413 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
+          <t>Chemical antagonist: which is right?</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Protamine neutralizes heparin — no receptor</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Always comparative — "compared to what?"</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Phase II — only ~25% move to Phase III</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Required proof of efficacy (thalidomide)</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>30</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>144</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Therapeutic window: which is right?</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>TI = TD₅₀ ÷ ED₅₀; narrow = careful dosing + blood levels</t>
+        </is>
+      </c>
+      <c r="G152" t="n">
+        <v>30</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>145</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Aspirin overdose: which is right?</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Sodium bicarbonate → alkaline urine → faster excretion</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Often first found in Phase IV — trials too small/short</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Adverse-event reporting system (voluntary + mandatory)</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Harm when dose/exposure exceeds the therapeutic range</t>
+        </is>
+      </c>
+      <c r="G153" t="n">
+        <v>30</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>146</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Most drugs’ molecular weight: which is right?</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Natural ligand unknown</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>~100–1000</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="G154" t="n">
+        <v>20</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>147</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Weak bonds vs covalent: which is right?</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+        </is>
+      </c>
+      <c r="G155" t="n">
+        <v>30</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>148</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>pKa: which is right?</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>20</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>149</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Ion trapping: which is right?</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Postmarketing surveillance — general prescribed population</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>30</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>150</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Intracellular receptors: which is right?</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
+        <v>30</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>151</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Gs / Gi / Gq: which is right?</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Phase II — only ~25% move to Phase III</t>
+        </is>
+      </c>
+      <c r="G159" t="n">
+        <v>20</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>152</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Gold-standard trial: which is right?</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>pH where ionized = nonionized</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Natural ligand unknown</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Brand name of acetaminophen</t>
+        </is>
+      </c>
+      <c r="G160" t="n">
+        <v>20</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>153</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
           <t>Orphan receptor: which is right?</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>Natural ligand unknown</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="D161" t="inlineStr">
         <is>
           <t>pH where ionized = nonionized</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E161" t="inlineStr">
         <is>
           <t>Randomized controlled trial</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F161" t="inlineStr">
         <is>
           <t>Brand name of acetaminophen</t>
         </is>
       </c>
-      <c r="G151" t="n">
+      <c r="G161" t="n">
         <v>20</v>
       </c>
-      <c r="H151" t="inlineStr">
+      <c r="H161" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>

<commit_message>
PA-level depth: textbook additions trimmed to what a PA needs (chemistry, molecular-biology and industry detail removed, repeats merged); decks carry lecture quick checks plus one question per part (L01 137→112, L02 124→104 slides); length gates (textbook share, bullet length, deck size) in the lecture standard; rules updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016g9Y35CWfsLvVnVtnzR7rF
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit1_L01.xlsx
+++ b/docs/sketch/kahoot/unit1_L01.xlsx
@@ -1589,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA161"/>
+  <dimension ref="A1:AA159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col width="12.5" customWidth="1" min="1" max="1"/>
@@ -7818,7 +7818,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Natural ligand unknown</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="G115" t="n">
@@ -9280,35 +9280,35 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Most drugs’ molecular weight: which is right?</t>
+          <t>Weak bonds vs covalent: which is right?</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Natural ligand unknown</t>
+          <t>Unintended, harmful response at normal therapeutic doses</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>~100–1000</t>
+          <t>Only free (unbound) drug is active and crosses membranes</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Min therapeutic → min toxic dose; more practical than TI</t>
         </is>
       </c>
       <c r="G154" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -9318,31 +9318,31 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Weak bonds vs covalent: which is right?</t>
+          <t>pKa: which is right?</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Unintended, harmful response at normal therapeutic doses</t>
+          <t>Brand name of acetaminophen</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Only free (unbound) drug is active and crosses membranes</t>
+          <t>Randomized controlled trial</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Weak = more selective; covalent = long-lasting (aspirin)</t>
+          <t>pH where ionized = nonionized</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Min therapeutic → min toxic dose; more practical than TI</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="G155" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
@@ -9356,31 +9356,31 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>pKa: which is right?</t>
+          <t>Ion trapping: which is right?</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Brand name of acetaminophen</t>
+          <t>Postmarketing surveillance — general prescribed population</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Randomized controlled trial</t>
+          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>pH where ionized = nonionized</t>
+          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+          <t>Usually poor BBB entry — better when meninges are inflamed</t>
         </is>
       </c>
       <c r="G156" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
@@ -9394,12 +9394,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Ion trapping: which is right?</t>
+          <t>Intracellular receptors: which is right?</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Postmarketing surveillance — general prescribed population</t>
+          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -9409,12 +9409,12 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Acids leave faster in alkaline urine; bases in acidic urine</t>
+          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Usually poor BBB entry — better when meninges are inflamed</t>
+          <t>Concentration giving 50% of Emax — standard measure of potency</t>
         </is>
       </c>
       <c r="G157" t="n">
@@ -9432,31 +9432,31 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Intracellular receptors: which is right?</t>
+          <t>Gs / Gi / Gq: which is right?</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Receptors · ion channels · enzymes · transporters · nucleic acids</t>
+          <t>pH where ionized = nonionized</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Nitroglycerin, propranolol, morphine — need higher oral doses</t>
+          <t>Warfarin, lithium, digoxin, phenytoin</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Steroids, thyroid, vitamin D; lag 30 min–hours, effect persists</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Concentration giving 50% of Emax — standard measure of potency</t>
+          <t>Phase II — only ~25% move to Phase III</t>
         </is>
       </c>
       <c r="G158" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
@@ -9470,7 +9470,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Gs / Gi / Gq: which is right?</t>
+          <t>Gold-standard trial: which is right?</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -9480,17 +9480,17 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Warfarin, lithium, digoxin, phenytoin</t>
+          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>↑ cAMP / ↓ cAMP / ↑ IP₃, DAG, Ca²⁺</t>
+          <t>Randomized controlled trial</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Phase II — only ~25% move to Phase III</t>
+          <t>Brand name of acetaminophen</t>
         </is>
       </c>
       <c r="G159" t="n">
@@ -9499,82 +9499,6 @@
       <c r="H159" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="n">
-        <v>152</v>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>Gold-standard trial: which is right?</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>pH where ionized = nonionized</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Natural ligand unknown</t>
-        </is>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Randomized controlled trial</t>
-        </is>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>Brand name of acetaminophen</t>
-        </is>
-      </c>
-      <c r="G160" t="n">
-        <v>20</v>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="n">
-        <v>153</v>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Orphan receptor: which is right?</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Natural ligand unknown</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>pH where ionized = nonionized</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Randomized controlled trial</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>Brand name of acetaminophen</t>
-        </is>
-      </c>
-      <c r="G161" t="n">
-        <v>20</v>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>